<commit_message>
Censor all geo information
</commit_message>
<xml_diff>
--- a/tests/fixtures/2021-2024 SDN Political-Related Sexual Violence Incident Data.xlsx
+++ b/tests/fixtures/2021-2024 SDN Political-Related Sexual Violence Incident Data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="72">
   <si>
     <t>Date</t>
   </si>
@@ -103,13 +103,7 @@
     <t>Khartoum State</t>
   </si>
   <si>
-    <t xml:space="preserve">(2) 25 km Precision </t>
-  </si>
-  <si>
-    <t>(6) Country</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(3) District, Communicipality or Commune </t>
+    <t>censored</t>
   </si>
   <si>
     <t>During Arrest or Detention</t>
@@ -661,53 +655,47 @@
       <c r="E2" t="s">
         <v>26</v>
       </c>
-      <c r="F2">
-        <v>14.3</v>
-      </c>
-      <c r="G2">
-        <v>33.5</v>
-      </c>
       <c r="H2" t="s">
         <v>29</v>
       </c>
       <c r="I2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J2" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" t="s">
         <v>36</v>
       </c>
-      <c r="K2" t="s">
-        <v>38</v>
-      </c>
       <c r="L2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M2" t="s">
         <v>41</v>
       </c>
-      <c r="M2" t="s">
-        <v>43</v>
-      </c>
       <c r="N2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O2" t="s">
+        <v>45</v>
+      </c>
+      <c r="P2" t="s">
         <v>47</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>49</v>
       </c>
-      <c r="Q2" t="s">
-        <v>51</v>
-      </c>
       <c r="R2" t="s">
+        <v>53</v>
+      </c>
+      <c r="S2" t="s">
         <v>55</v>
-      </c>
-      <c r="S2" t="s">
-        <v>57</v>
       </c>
       <c r="T2">
         <v>8</v>
       </c>
       <c r="V2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="W2" s="1">
         <v>45450</v>
@@ -729,53 +717,47 @@
       <c r="E3" t="s">
         <v>27</v>
       </c>
-      <c r="F3">
-        <v>15.5</v>
-      </c>
-      <c r="G3">
-        <v>32.4</v>
-      </c>
       <c r="H3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I3" t="s">
         <v>27</v>
       </c>
       <c r="J3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="K3" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3" t="s">
         <v>39</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>41</v>
       </c>
-      <c r="M3" t="s">
-        <v>43</v>
-      </c>
       <c r="N3" t="s">
+        <v>44</v>
+      </c>
+      <c r="O3" t="s">
         <v>46</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>48</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>50</v>
       </c>
-      <c r="Q3" t="s">
-        <v>52</v>
-      </c>
       <c r="R3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="S3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="T3">
         <v>3</v>
       </c>
       <c r="V3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="W3" s="1">
         <v>44718</v>
@@ -797,53 +779,47 @@
       <c r="E4" t="s">
         <v>28</v>
       </c>
-      <c r="F4">
-        <v>15.6</v>
-      </c>
-      <c r="G4">
-        <v>32.5</v>
-      </c>
       <c r="H4" t="s">
         <v>29</v>
       </c>
       <c r="I4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K4" t="s">
         <v>36</v>
       </c>
-      <c r="K4" t="s">
-        <v>38</v>
-      </c>
       <c r="L4" t="s">
+        <v>39</v>
+      </c>
+      <c r="M4" t="s">
         <v>41</v>
       </c>
-      <c r="M4" t="s">
-        <v>43</v>
-      </c>
       <c r="N4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O4" t="s">
         <v>46</v>
       </c>
-      <c r="O4" t="s">
-        <v>48</v>
-      </c>
       <c r="P4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="Q4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="R4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="S4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T4">
         <v>1</v>
       </c>
       <c r="V4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="W4" s="1">
         <v>44718</v>
@@ -865,53 +841,47 @@
       <c r="E5" t="s">
         <v>28</v>
       </c>
-      <c r="F5">
-        <v>15.6</v>
-      </c>
-      <c r="G5">
-        <v>32.4</v>
-      </c>
       <c r="H5" t="s">
         <v>29</v>
       </c>
       <c r="I5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="K5" t="s">
+        <v>37</v>
+      </c>
+      <c r="L5" t="s">
         <v>39</v>
       </c>
-      <c r="L5" t="s">
-        <v>41</v>
-      </c>
       <c r="M5" t="s">
+        <v>42</v>
+      </c>
+      <c r="N5" t="s">
         <v>44</v>
       </c>
-      <c r="N5" t="s">
-        <v>46</v>
-      </c>
       <c r="O5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="Q5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R5" t="s">
+        <v>53</v>
+      </c>
+      <c r="S5" t="s">
         <v>55</v>
-      </c>
-      <c r="S5" t="s">
-        <v>57</v>
       </c>
       <c r="T5">
         <v>2</v>
       </c>
       <c r="V5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="W5" s="1">
         <v>44717</v>
@@ -933,53 +903,47 @@
       <c r="E6" t="s">
         <v>28</v>
       </c>
-      <c r="F6">
-        <v>15.6</v>
-      </c>
-      <c r="G6">
-        <v>32.4</v>
-      </c>
       <c r="H6" t="s">
         <v>29</v>
       </c>
       <c r="I6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L6" t="s">
+        <v>39</v>
+      </c>
+      <c r="M6" t="s">
         <v>41</v>
       </c>
-      <c r="M6" t="s">
-        <v>43</v>
-      </c>
       <c r="N6" t="s">
+        <v>44</v>
+      </c>
+      <c r="O6" t="s">
         <v>46</v>
       </c>
-      <c r="O6" t="s">
-        <v>48</v>
-      </c>
       <c r="P6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="Q6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="R6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="S6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T6">
         <v>1</v>
       </c>
       <c r="V6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="W6" s="1">
         <v>44614</v>
@@ -1001,53 +965,47 @@
       <c r="E7" t="s">
         <v>28</v>
       </c>
-      <c r="F7">
-        <v>15.6</v>
-      </c>
-      <c r="G7">
-        <v>32.3</v>
-      </c>
       <c r="H7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K7" t="s">
+        <v>38</v>
+      </c>
+      <c r="L7" t="s">
         <v>40</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>42</v>
       </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>44</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>46</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
         <v>48</v>
       </c>
-      <c r="P7" t="s">
+      <c r="Q7" t="s">
         <v>50</v>
       </c>
-      <c r="Q7" t="s">
-        <v>52</v>
-      </c>
       <c r="R7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="S7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="T7">
         <v>1</v>
       </c>
       <c r="V7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="W7" s="1">
         <v>44617</v>
@@ -1069,12 +1027,6 @@
       <c r="E8" t="s">
         <v>28</v>
       </c>
-      <c r="F8">
-        <v>15.6</v>
-      </c>
-      <c r="G8">
-        <v>32.5</v>
-      </c>
       <c r="H8" t="s">
         <v>29</v>
       </c>
@@ -1082,40 +1034,40 @@
         <v>27</v>
       </c>
       <c r="J8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L8" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M8" t="s">
+        <v>43</v>
+      </c>
+      <c r="N8" t="s">
+        <v>44</v>
+      </c>
+      <c r="O8" t="s">
         <v>45</v>
       </c>
-      <c r="N8" t="s">
-        <v>46</v>
-      </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
         <v>47</v>
       </c>
-      <c r="P8" t="s">
-        <v>49</v>
-      </c>
       <c r="Q8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="R8" t="s">
+        <v>54</v>
+      </c>
+      <c r="S8" t="s">
         <v>56</v>
-      </c>
-      <c r="S8" t="s">
-        <v>58</v>
       </c>
       <c r="T8">
         <v>3</v>
       </c>
       <c r="V8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="W8" s="1">
         <v>44578</v>
@@ -1137,12 +1089,6 @@
       <c r="E9" t="s">
         <v>28</v>
       </c>
-      <c r="F9">
-        <v>15.6</v>
-      </c>
-      <c r="G9">
-        <v>32.5</v>
-      </c>
       <c r="H9" t="s">
         <v>29</v>
       </c>
@@ -1150,40 +1096,40 @@
         <v>27</v>
       </c>
       <c r="J9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L9" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="N9" t="s">
+        <v>44</v>
+      </c>
+      <c r="O9" t="s">
         <v>46</v>
       </c>
-      <c r="O9" t="s">
-        <v>48</v>
-      </c>
       <c r="P9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="Q9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="R9" t="s">
+        <v>54</v>
+      </c>
+      <c r="S9" t="s">
         <v>56</v>
-      </c>
-      <c r="S9" t="s">
-        <v>58</v>
       </c>
       <c r="T9">
         <v>13</v>
       </c>
       <c r="V9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="W9" s="1">
         <v>44578</v>
@@ -1205,12 +1151,6 @@
       <c r="E10" t="s">
         <v>28</v>
       </c>
-      <c r="F10">
-        <v>15.6</v>
-      </c>
-      <c r="G10">
-        <v>32.5</v>
-      </c>
       <c r="H10" t="s">
         <v>29</v>
       </c>
@@ -1218,40 +1158,40 @@
         <v>27</v>
       </c>
       <c r="J10" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L10" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="N10" t="s">
+        <v>44</v>
+      </c>
+      <c r="O10" t="s">
         <v>46</v>
       </c>
-      <c r="O10" t="s">
-        <v>48</v>
-      </c>
       <c r="P10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="Q10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="R10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="S10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="T10">
         <v>30</v>
       </c>
       <c r="V10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="W10" s="1">
         <v>44578</v>
@@ -1273,53 +1213,47 @@
       <c r="E11" t="s">
         <v>28</v>
       </c>
-      <c r="F11">
-        <v>15.6</v>
-      </c>
-      <c r="G11">
-        <v>32.5</v>
-      </c>
       <c r="H11" t="s">
         <v>29</v>
       </c>
       <c r="I11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J11" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L11" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M11" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="N11" t="s">
+        <v>44</v>
+      </c>
+      <c r="O11" t="s">
         <v>46</v>
       </c>
-      <c r="O11" t="s">
+      <c r="P11" t="s">
         <v>48</v>
       </c>
-      <c r="P11" t="s">
+      <c r="Q11" t="s">
         <v>50</v>
       </c>
-      <c r="Q11" t="s">
-        <v>52</v>
-      </c>
       <c r="R11" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="S11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="T11">
         <v>1</v>
       </c>
       <c r="V11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="W11" s="1">
         <v>44578</v>
@@ -1341,12 +1275,6 @@
       <c r="E12" t="s">
         <v>28</v>
       </c>
-      <c r="F12">
-        <v>15.6</v>
-      </c>
-      <c r="G12">
-        <v>32.5</v>
-      </c>
       <c r="H12" t="s">
         <v>29</v>
       </c>
@@ -1354,40 +1282,40 @@
         <v>27</v>
       </c>
       <c r="J12" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="N12" t="s">
+        <v>44</v>
+      </c>
+      <c r="O12" t="s">
         <v>46</v>
       </c>
-      <c r="O12" t="s">
-        <v>48</v>
-      </c>
       <c r="P12" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="Q12" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="R12" t="s">
+        <v>54</v>
+      </c>
+      <c r="S12" t="s">
         <v>56</v>
-      </c>
-      <c r="S12" t="s">
-        <v>58</v>
       </c>
       <c r="T12">
         <v>13</v>
       </c>
       <c r="V12" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="W12" s="1">
         <v>44578</v>
@@ -1409,53 +1337,47 @@
       <c r="E13" t="s">
         <v>28</v>
       </c>
-      <c r="F13">
-        <v>15.6</v>
-      </c>
-      <c r="G13">
-        <v>32.5</v>
-      </c>
       <c r="H13" t="s">
         <v>29</v>
       </c>
       <c r="I13" t="s">
+        <v>33</v>
+      </c>
+      <c r="J13" t="s">
         <v>35</v>
       </c>
-      <c r="J13" t="s">
-        <v>37</v>
-      </c>
       <c r="K13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L13" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M13" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="N13" t="s">
+        <v>44</v>
+      </c>
+      <c r="O13" t="s">
         <v>46</v>
       </c>
-      <c r="O13" t="s">
-        <v>48</v>
-      </c>
       <c r="P13" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="Q13" t="s">
+        <v>52</v>
+      </c>
+      <c r="R13" t="s">
         <v>54</v>
       </c>
-      <c r="R13" t="s">
+      <c r="S13" t="s">
         <v>56</v>
-      </c>
-      <c r="S13" t="s">
-        <v>58</v>
       </c>
       <c r="T13">
         <v>6</v>
       </c>
       <c r="V13" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="W13" s="1">
         <v>44578</v>

</xml_diff>